<commit_message>
docs: remover textos de preenchimento e revisar evidências da Etapa 3
Remove orientações de envio ao Canvas, campos genéricos e instruções editoriais. Mantém fatos de implementação, autoria e limites da validação. Preserva fórmulas e metas do Balanced Scorecard.
</commit_message>
<xml_diff>
--- a/planilhas/Balanced_Scorecard.xlsx
+++ b/planilhas/Balanced_Scorecard.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financeira" sheetId="1" r:id="Rfb647f7ffbc842ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="2" r:id="R5e4adc8db1634397"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Processos internos" sheetId="3" r:id="Rb2be32ca233b4846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aprendizado" sheetId="4" r:id="R776ac6c441ec49ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financeira" sheetId="1" r:id="Re59bd20c16864120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="2" r:id="Rab8f6ebac7ce4370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Processos internos" sheetId="3" r:id="R61de66b733974f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aprendizado" sheetId="4" r:id="Rb613cac20f424114"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Metas propostas para os 12 meses do piloto. Preencher resultados reais nas células amarelas.</x:v>
+        <x:v>Metas propostas para os 12 meses do piloto. Resultados operacionais sem medição.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -469,7 +469,7 @@
         <x:v>Periodicidade</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Responsável proposto</x:v>
+        <x:v>Função responsável</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>Iniciativa</x:v>
@@ -500,7 +500,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>Comercial / a designar</x:v>
+        <x:v>Comercial</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
         <x:v>Validar preço e conquistar 20 assinantes.</x:v>
@@ -531,7 +531,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>Comercial / a designar</x:v>
+        <x:v>Comercial</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>Medir gastos comerciais e conversões por canal.</x:v>
@@ -562,7 +562,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Financeiro / a designar</x:v>
+        <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="J8" s="7" t="str">
         <x:v>Revisar fluxo e formar reserva antes de expandir.</x:v>
@@ -688,7 +688,7 @@
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>Resultados reais e responsáveis individuais ainda não informados. Data de elaboração: 21/10/2026.</x:v>
+        <x:v>Responsabilidades organizadas por função. Data de elaboração: 21/10/2026.</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
@@ -767,7 +767,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Metas propostas para os 12 meses do piloto. Preencher resultados reais nas células amarelas.</x:v>
+        <x:v>Metas propostas para os 12 meses do piloto. Resultados operacionais sem medição.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -817,7 +817,7 @@
         <x:v>Periodicidade</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Responsável proposto</x:v>
+        <x:v>Função responsável</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>Iniciativa</x:v>
@@ -848,7 +848,7 @@
         <x:v>Por entrega</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>Atendimento / a designar</x:v>
+        <x:v>Atendimento</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
         <x:v>Aplicar pesquisa após diagnóstico.</x:v>
@@ -879,7 +879,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>Comercial / a designar</x:v>
+        <x:v>Comercial</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>Revisar causas de cancelamento e plano de ação.</x:v>
@@ -910,7 +910,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Consultoria / a designar</x:v>
+        <x:v>Consultoria</x:v>
       </x:c>
       <x:c r="J8" s="7" t="str">
         <x:v>Registrar prazo acordado e data de liberação.</x:v>
@@ -1036,7 +1036,7 @@
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>Resultados reais e responsáveis individuais ainda não informados. Data de elaboração: 21/10/2026.</x:v>
+        <x:v>Responsabilidades organizadas por função. Data de elaboração: 21/10/2026.</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
@@ -1115,7 +1115,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Metas propostas para os 12 meses do piloto. Preencher resultados reais nas células amarelas.</x:v>
+        <x:v>Metas propostas para os 12 meses do piloto. Resultados operacionais sem medição.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1165,7 +1165,7 @@
         <x:v>Periodicidade</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Responsável proposto</x:v>
+        <x:v>Função responsável</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>Iniciativa</x:v>
@@ -1196,7 +1196,7 @@
         <x:v>Por sprint</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>Backend / a designar</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
         <x:v>Implementar casos positivos, negativos e insuficientes.</x:v>
@@ -1227,7 +1227,7 @@
         <x:v>Por sprint</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>Qualidade / a designar</x:v>
+        <x:v>Qualidade</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>Testar bloqueios e auditoria de revisão.</x:v>
@@ -1258,7 +1258,7 @@
         <x:v>Por entrega</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Consultoria / a designar</x:v>
+        <x:v>Consultoria</x:v>
       </x:c>
       <x:c r="J8" s="7" t="str">
         <x:v>Cronometrar revisão completa no piloto.</x:v>
@@ -1384,7 +1384,7 @@
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>Resultados reais e responsáveis individuais ainda não informados. Data de elaboração: 21/10/2026.</x:v>
+        <x:v>Responsabilidades organizadas por função. Data de elaboração: 21/10/2026.</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
@@ -1463,7 +1463,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Metas propostas para os 12 meses do piloto. Preencher resultados reais nas células amarelas.</x:v>
+        <x:v>Metas propostas para os 12 meses do piloto. Resultados operacionais sem medição.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1513,7 +1513,7 @@
         <x:v>Periodicidade</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Responsável proposto</x:v>
+        <x:v>Função responsável</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>Iniciativa</x:v>
@@ -1544,7 +1544,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>Equipe / a designar</x:v>
+        <x:v>Equipe</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
         <x:v>Estudar Flask, redes e testes; registrar evidência.</x:v>
@@ -1575,7 +1575,7 @@
         <x:v>Por sprint</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>Equipe / a designar</x:v>
+        <x:v>Equipe</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>Cada integrante assumir issue e entregar mudança real.</x:v>
@@ -1606,7 +1606,7 @@
         <x:v>Mensal</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Equipe / a designar</x:v>
+        <x:v>Equipe</x:v>
       </x:c>
       <x:c r="J8" s="7" t="str">
         <x:v>Registrar revisão e decisão técnica em PR.</x:v>
@@ -1732,7 +1732,7 @@
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>Resultados reais e responsáveis individuais ainda não informados. Data de elaboração: 21/10/2026.</x:v>
+        <x:v>Responsabilidades organizadas por função. Data de elaboração: 21/10/2026.</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>

</xml_diff>